<commit_message>
changes with app.js file
</commit_message>
<xml_diff>
--- a/MOCK_DATAa.xlsx
+++ b/MOCK_DATAa.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uwacloud-my.sharepoint.com/personal/upundeer_univ-wea_com/Documents/Desktop/last_mile/backend/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uwacloud-my.sharepoint.com/personal/upundeer_univ-wea_com/Documents/Desktop/backend/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="148" documentId="11_46B11697F22F9737756696BF9120C9AEE7B8F16E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{18D5F754-2F73-4632-B20D-95551E953638}"/>
+  <xr:revisionPtr revIDLastSave="154" documentId="11_46B11697F22F9737756696BF9120C9AEE7B8F16E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{13EE0A17-2E72-4AF3-B575-D8EDE1FC42F1}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="1152" yWindow="1152" windowWidth="17280" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1848" yWindow="1848" windowWidth="17280" windowHeight="9420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
@@ -185,6 +185,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -482,6 +486,7 @@
     <col min="6" max="6" width="10.33203125" style="2" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8.88671875" style="1"/>
     <col min="8" max="8" width="11.33203125" customWidth="1"/>
+    <col min="10" max="10" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.3">
@@ -509,7 +514,7 @@
       <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
     </row>
@@ -540,7 +545,7 @@
       </c>
       <c r="I2" s="4"/>
       <c r="J2" s="1">
-        <v>0.76041666666666663</v>
+        <v>1.6666666666666666E-2</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
@@ -570,7 +575,7 @@
       </c>
       <c r="I3" s="4"/>
       <c r="J3" s="1">
-        <v>0.76388888888888884</v>
+        <v>1.8749999999999999E-2</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">

</xml_diff>